<commit_message>
added web features 3
</commit_message>
<xml_diff>
--- a/templates/baselines/TansiMotorHiring.xlsx
+++ b/templates/baselines/TansiMotorHiring.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E30"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -654,9 +654,264 @@
         <v>aniketkumarsharma03@gmail.com</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>2026-02-26T10:57:56-05:00</v>
+      </c>
+      <c r="B16" t="str">
+        <v>▄︻デU̷D̷A̷Y̷ ̷F̷O̷X̷══━一</v>
+      </c>
+      <c r="C16" t="str">
+        <v>8618958815</v>
+      </c>
+      <c r="D16" t="str">
+        <v>DeliveryExecutives</v>
+      </c>
+      <c r="E16" t="str">
+        <v>uk15062004@gmail.com</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>2026-02-26T10:56:47-05:00</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Somanath</v>
+      </c>
+      <c r="C17" t="str">
+        <v>9019348859</v>
+      </c>
+      <c r="D17" t="str">
+        <v>ServiceAdvisors</v>
+      </c>
+      <c r="E17" t="str">
+        <v>somanathbuhler@gmail.com</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>2026-02-26T10:49:57-05:00</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Deepak Harsha</v>
+      </c>
+      <c r="C18" t="str">
+        <v>8892444994</v>
+      </c>
+      <c r="D18" t="str">
+        <v>SalesExecutives</v>
+      </c>
+      <c r="E18" t="str">
+        <v>harshadeepak312@gmail.com</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>2026-02-26T10:49:53-05:00</v>
+      </c>
+      <c r="B19" t="str">
+        <v>♡....</v>
+      </c>
+      <c r="C19" t="str">
+        <v>9901497723</v>
+      </c>
+      <c r="D19" t="str">
+        <v>SalesExecutives</v>
+      </c>
+      <c r="E19" t="str">
+        <v>salmankhan110bob@gmail.com</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>2026-02-26T10:43:17-05:00</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Prashanth K R</v>
+      </c>
+      <c r="C20" t="str">
+        <v>7996268862</v>
+      </c>
+      <c r="D20" t="str">
+        <v>BillingExecutives</v>
+      </c>
+      <c r="E20" t="str">
+        <v>gowdaprashi16@gmail.com</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>2026-02-26T10:37:57-05:00</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Siddu R</v>
+      </c>
+      <c r="C21" t="str">
+        <v>9902636962</v>
+      </c>
+      <c r="D21" t="str">
+        <v>ServiceManager</v>
+      </c>
+      <c r="E21" t="str">
+        <v>sadashivakalyani@gmail.com</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>2026-02-26T10:36:46-05:00</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Mssuresh</v>
+      </c>
+      <c r="C22" t="str">
+        <v>8792872031</v>
+      </c>
+      <c r="D22" t="str">
+        <v>SparePartsSupervisors</v>
+      </c>
+      <c r="E22" t="str">
+        <v>mssuresh123@gmail.com</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>2026-02-26T10:29:18-05:00</v>
+      </c>
+      <c r="B23" t="str">
+        <v>V Siva Mohan</v>
+      </c>
+      <c r="C23" t="str">
+        <v>9502103518</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Cashiers</v>
+      </c>
+      <c r="E23" t="str">
+        <v>vrsm1981@gmail.com</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>2026-02-26T10:13:27-05:00</v>
+      </c>
+      <c r="B24" t="str">
+        <v>🅥🅘🅝🅐🅨 🅚🅤🅜🅐🅡</v>
+      </c>
+      <c r="C24" t="str">
+        <v>7993157074</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Cashiers</v>
+      </c>
+      <c r="E24" t="str">
+        <v>chithulurivinaykumar@gmail.com</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>2026-02-26T11:35:57-05:00</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Prathap</v>
+      </c>
+      <c r="C25" t="str">
+        <v>9742385253</v>
+      </c>
+      <c r="D25" t="str">
+        <v>BillingExecutives</v>
+      </c>
+      <c r="E25" t="str">
+        <v>prathapo713@gmail.com</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>2026-02-26T11:33:46-05:00</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Dinesh Vk</v>
+      </c>
+      <c r="C26" t="str">
+        <v>7760666352</v>
+      </c>
+      <c r="D26" t="str">
+        <v>ServiceAdvisors</v>
+      </c>
+      <c r="E26" t="str">
+        <v>661dinesh.k@gmail.com</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>2026-02-26T11:16:54-05:00</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Kumar Tan</v>
+      </c>
+      <c r="C27" t="str">
+        <v>9738225644</v>
+      </c>
+      <c r="D27" t="str">
+        <v>ServiceManager</v>
+      </c>
+      <c r="E27" t="str">
+        <v>kumartan003@gmail.com</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>2026-02-26T11:15:16-05:00</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Suresh Suree</v>
+      </c>
+      <c r="C28" t="str">
+        <v>9901078053</v>
+      </c>
+      <c r="D28" t="str">
+        <v>ServiceManager</v>
+      </c>
+      <c r="E28" t="str">
+        <v>sureesuresh14@gmail.com</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>2026-02-26T11:06:50-05:00</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Amaravathi Nani</v>
+      </c>
+      <c r="C29" t="str">
+        <v>6374686459</v>
+      </c>
+      <c r="D29" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E29" t="str">
+        <v>nani3456782@gmail.com</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-02-26T11:02:15-05:00</v>
+      </c>
+      <c r="B30" t="str">
+        <v>ರಾಕೇಶ್ ರಾಖಿ</v>
+      </c>
+      <c r="C30" t="str">
+        <v>8861021266</v>
+      </c>
+      <c r="D30" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E30" t="str">
+        <v>rakeshrbpet@gmail.com</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added web features 5
</commit_message>
<xml_diff>
--- a/templates/baselines/TansiMotorHiring.xlsx
+++ b/templates/baselines/TansiMotorHiring.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -909,9 +909,468 @@
         <v>rakeshrbpet@gmail.com</v>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-02-26T11:40:28-05:00</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Salim Khan</v>
+      </c>
+      <c r="C31" t="str">
+        <v>9035724459</v>
+      </c>
+      <c r="D31" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E31" t="str">
+        <v>salimsallukhan1993@gmail.com</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>2026-02-26T23:43:41-05:00</v>
+      </c>
+      <c r="B32" t="str">
+        <v>⁴⁰★Mr.Devil★⁷²</v>
+      </c>
+      <c r="C32" t="str">
+        <v>6363857412</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Cashiers</v>
+      </c>
+      <c r="E32" t="str">
+        <v>manju5008d@gmail.com</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>2026-02-26T23:29:12-05:00</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Pavan Kumar</v>
+      </c>
+      <c r="C33" t="str">
+        <v>8885891998</v>
+      </c>
+      <c r="D33" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E33" t="str">
+        <v>pavannaik9849@gmail.com</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>2026-02-26T22:54:00-05:00</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Mohammed Ali</v>
+      </c>
+      <c r="C34" t="str">
+        <v>8904884463</v>
+      </c>
+      <c r="D34" t="str">
+        <v>SparePartsSupervisors</v>
+      </c>
+      <c r="E34" t="str">
+        <v>mohammedaamire78@gmail.com</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>2026-02-26T22:34:27-05:00</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Sibgathulla Sharieff T.H</v>
+      </c>
+      <c r="C35" t="str">
+        <v>9844730433</v>
+      </c>
+      <c r="D35" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E35" t="str">
+        <v>sharieff4uall97@gmail.com</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>2026-02-26T22:32:43-05:00</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Ganga Raj  Gangu</v>
+      </c>
+      <c r="C36" t="str">
+        <v>7204414982</v>
+      </c>
+      <c r="D36" t="str">
+        <v>DeliveryExecutives</v>
+      </c>
+      <c r="E36" t="str">
+        <v>gangaraju.1998.2016@gmail.com</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>2026-02-26T22:19:43-05:00</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Antony Ruban Maharaj</v>
+      </c>
+      <c r="C37" t="str">
+        <v>9632251007</v>
+      </c>
+      <c r="D37" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E37" t="str">
+        <v>maharaj.antony@gmail.com</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>2026-02-26T22:01:06-05:00</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Amar Nath</v>
+      </c>
+      <c r="C38" t="str">
+        <v>8095229450</v>
+      </c>
+      <c r="D38" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E38" t="str">
+        <v>my143amar@gmail.comm</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>2026-02-26T21:20:04-05:00</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Akshata Ellamasi</v>
+      </c>
+      <c r="C39" t="str">
+        <v>8431069837</v>
+      </c>
+      <c r="D39" t="str">
+        <v>SalesExecutives</v>
+      </c>
+      <c r="E39" t="str">
+        <v>akshatakiran8@gmail.com</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>2026-02-26T20:14:10-05:00</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Hemanth Nagishetty</v>
+      </c>
+      <c r="C40" t="str">
+        <v>9886190419</v>
+      </c>
+      <c r="D40" t="str">
+        <v>ServiceManager</v>
+      </c>
+      <c r="E40" t="str">
+        <v>nhemanth92@gmail.com</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>2026-02-26T20:09:07-05:00</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Bharath</v>
+      </c>
+      <c r="C41" t="str">
+        <v>9916567868</v>
+      </c>
+      <c r="D41" t="str">
+        <v>ServiceManager</v>
+      </c>
+      <c r="E41" t="str">
+        <v>bhrthbabu6@gmail.com</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>2026-02-26T16:05:48-05:00</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Santosh</v>
+      </c>
+      <c r="C42" t="str">
+        <v>9740857979</v>
+      </c>
+      <c r="D42" t="str">
+        <v>ServiceAdvisors</v>
+      </c>
+      <c r="E42" t="str">
+        <v>santoshmhosur1995@gmail.com</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>2026-02-26T15:44:58-05:00</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Sarfaraz Nawaz</v>
+      </c>
+      <c r="C43" t="str">
+        <v>9740899465</v>
+      </c>
+      <c r="D43" t="str">
+        <v>SalesExecutives</v>
+      </c>
+      <c r="E43" t="str">
+        <v>max.nawaz@gmail.com</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>2026-02-26T15:43:30-05:00</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Antony</v>
+      </c>
+      <c r="C44" t="str">
+        <v>9900583777</v>
+      </c>
+      <c r="D44" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E44" t="str">
+        <v>shojyantony@hmail.com</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>2026-02-26T14:46:42-05:00</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Santhosh Gowda</v>
+      </c>
+      <c r="C45" t="str">
+        <v>7259880716</v>
+      </c>
+      <c r="D45" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E45" t="str">
+        <v>santhoshaur@gmail.com</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>2026-02-26T14:10:50-05:00</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Syed Sameer S</v>
+      </c>
+      <c r="C46" t="str">
+        <v>9019908853</v>
+      </c>
+      <c r="D46" t="str">
+        <v>BillingExecutives</v>
+      </c>
+      <c r="E46" t="str">
+        <v>samsameer1103@gmail.com</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>2026-02-26T14:00:20-05:00</v>
+      </c>
+      <c r="B47" t="str">
+        <v>&lt;꧁༺$Elva Thrile༻꧂&gt;</v>
+      </c>
+      <c r="C47" t="str">
+        <v>8073561794</v>
+      </c>
+      <c r="D47" t="str">
+        <v>SalesExecutives</v>
+      </c>
+      <c r="E47" t="str">
+        <v>anusreeselva2014@gmail.com</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>2026-02-26T13:55:49-05:00</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Nagaraja N</v>
+      </c>
+      <c r="C48" t="str">
+        <v>9686325546</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Cashiers</v>
+      </c>
+      <c r="E48" t="str">
+        <v>nagkimg2410@gmail.com</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>2026-02-26T13:55:36-05:00</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Vinod Sarashetti</v>
+      </c>
+      <c r="C49" t="str">
+        <v>8970842145</v>
+      </c>
+      <c r="D49" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E49" t="str">
+        <v>vsarashetti09@gmail.com</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>2026-02-26T13:45:29-05:00</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Darshan Patgar</v>
+      </c>
+      <c r="C50" t="str">
+        <v>8971234659</v>
+      </c>
+      <c r="D50" t="str">
+        <v>BillingExecutives</v>
+      </c>
+      <c r="E50" t="str">
+        <v>darshanpatgar6362@gmail.com</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>2026-02-26T13:42:10-05:00</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Amarnath</v>
+      </c>
+      <c r="C51" t="str">
+        <v>7022670892</v>
+      </c>
+      <c r="D51" t="str">
+        <v>SalesExecutives</v>
+      </c>
+      <c r="E51" t="str">
+        <v>chaitranishchai@gmail.com</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>2026-02-26T13:34:26-05:00</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Deepak</v>
+      </c>
+      <c r="C52" t="str">
+        <v>9844220769</v>
+      </c>
+      <c r="D52" t="str">
+        <v>SalesManager</v>
+      </c>
+      <c r="E52" t="str">
+        <v>deepakgowda.m7@gmail.com</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>2026-02-26T13:33:54-05:00</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Shoeb</v>
+      </c>
+      <c r="C53" t="str">
+        <v>8431464421</v>
+      </c>
+      <c r="D53" t="str">
+        <v>SparePartsSupervisors</v>
+      </c>
+      <c r="E53" t="str">
+        <v>shoebshaik903@gmail.com</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>2026-02-26T12:54:08-05:00</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Kiran</v>
+      </c>
+      <c r="C54" t="str">
+        <v>9620430310</v>
+      </c>
+      <c r="D54" t="str">
+        <v>ServiceAdvisors</v>
+      </c>
+      <c r="E54" t="str">
+        <v>kiranvarne1234@gmail.com</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>2026-02-26T12:23:48-05:00</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Bhoomika</v>
+      </c>
+      <c r="C55" t="str">
+        <v>9380622780</v>
+      </c>
+      <c r="D55" t="str">
+        <v>BillingExecutives</v>
+      </c>
+      <c r="E55" t="str">
+        <v>b30040483@gmail.com</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>2026-02-26T12:13:16-05:00</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Karthick Gowda Karthik</v>
+      </c>
+      <c r="C56" t="str">
+        <v>7483021215</v>
+      </c>
+      <c r="D56" t="str">
+        <v>SparePartsSupervisors</v>
+      </c>
+      <c r="E56" t="str">
+        <v>bettegowdalalithag@gmail.com</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>2026-02-26T11:55:10-05:00</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Amaranatha V H</v>
+      </c>
+      <c r="C57" t="str">
+        <v>8747988272</v>
+      </c>
+      <c r="D57" t="str">
+        <v>SparePartsSupervisors</v>
+      </c>
+      <c r="E57" t="str">
+        <v>madhuamar272@gmail.com</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E30"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>